<commit_message>
fix: Use `citizens_per_class` or `places_of_employment` for income distributions
The initialization of `income_distributions` only considered the
`citizens_per_class` input data and did not contain a switch to use the
`places_of_employment` whenever the flag `citizens` is False.

That inconsistency is addressed in this patch by moving the
initialization of the `income_distributions` array into a separate
function to which we either supply the `citizens_per_class` or
`places_of_employment` data depending on the context.
</commit_message>
<xml_diff>
--- a/tests/vlaanderen/reference/resultaten/werk/concurrentie/arbeidsplaatsen/restdag/Ontpl_conc_Auto.xlsx
+++ b/tests/vlaanderen/reference/resultaten/werk/concurrentie/arbeidsplaatsen/restdag/Ontpl_conc_Auto.xlsx
@@ -385,16 +385,16 @@
         <v>1</v>
       </c>
       <c r="B2">
-        <v>0.4532370357302815</v>
+        <v>1.531506941692202</v>
       </c>
       <c r="C2">
-        <v>0.6303542376453837</v>
+        <v>1.002349831076548</v>
       </c>
       <c r="D2">
-        <v>0.7092559956622544</v>
+        <v>0.5809953305784216</v>
       </c>
       <c r="E2">
-        <v>0.7506371350073703</v>
+        <v>0.4038877269654029</v>
       </c>
     </row>
     <row r="3" spans="1:5">
@@ -402,16 +402,16 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>0.4823481996652292</v>
+        <v>0.9143015430915289</v>
       </c>
       <c r="C3">
-        <v>0.6453361537028188</v>
+        <v>0.6626040320786434</v>
       </c>
       <c r="D3">
-        <v>0.7171446371773404</v>
+        <v>0.6058032171232366</v>
       </c>
       <c r="E3">
-        <v>0.7560526663458433</v>
+        <v>0.575585512586713</v>
       </c>
     </row>
     <row r="4" spans="1:5">
@@ -419,16 +419,16 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>0.4358399287341901</v>
+        <v>1.063143573529856</v>
       </c>
       <c r="C4">
-        <v>0.6212544359327956</v>
+        <v>0.8056689105991625</v>
       </c>
       <c r="D4">
-        <v>0.7103663845345167</v>
+        <v>0.5775984918460773</v>
       </c>
       <c r="E4">
-        <v>0.7512958322845921</v>
+        <v>0.4732372905674737</v>
       </c>
     </row>
     <row r="5" spans="1:5">
@@ -436,16 +436,16 @@
         <v>4</v>
       </c>
       <c r="B5">
-        <v>0.5508185575131226</v>
+        <v>0.1372783092254067</v>
       </c>
       <c r="C5">
-        <v>0.7087126653779002</v>
+        <v>0.1777267055591638</v>
       </c>
       <c r="D5">
-        <v>0.7497438449623276</v>
+        <v>0.1868556641469578</v>
       </c>
       <c r="E5">
-        <v>0.7843231854640947</v>
+        <v>0.1966878576550826</v>
       </c>
     </row>
     <row r="6" spans="1:5">
@@ -453,16 +453,16 @@
         <v>5</v>
       </c>
       <c r="B6">
-        <v>0.5359501924988801</v>
+        <v>0.5900184310518355</v>
       </c>
       <c r="C6">
-        <v>0.6926616539226804</v>
+        <v>0.6000310092678657</v>
       </c>
       <c r="D6">
-        <v>0.7442507980091263</v>
+        <v>0.7022854430926124</v>
       </c>
       <c r="E6">
-        <v>0.7814385392731652</v>
+        <v>0.8913980626552414</v>
       </c>
     </row>
     <row r="7" spans="1:5">
@@ -470,16 +470,16 @@
         <v>6</v>
       </c>
       <c r="B7">
-        <v>0.5704041248505743</v>
+        <v>1.083767837216091</v>
       </c>
       <c r="C7">
-        <v>0.7150384956991823</v>
+        <v>0.6792865709142233</v>
       </c>
       <c r="D7">
-        <v>0.7634258695380866</v>
+        <v>0.659322341873802</v>
       </c>
       <c r="E7">
-        <v>0.7894287252199673</v>
+        <v>0.6249644074658074</v>
       </c>
     </row>
     <row r="8" spans="1:5">
@@ -487,16 +487,16 @@
         <v>7</v>
       </c>
       <c r="B8">
-        <v>0.3440101165016323</v>
+        <v>0.0859764123537332</v>
       </c>
       <c r="C8">
-        <v>0.5363111047676458</v>
+        <v>0.134199924181154</v>
       </c>
       <c r="D8">
-        <v>0.6528399286774035</v>
+        <v>0.1631604194659894</v>
       </c>
       <c r="E8">
-        <v>0.7281542421987869</v>
+        <v>0.1819832800879447</v>
       </c>
     </row>
     <row r="9" spans="1:5">
@@ -504,16 +504,16 @@
         <v>8</v>
       </c>
       <c r="B9">
-        <v>0.5618944707293718</v>
+        <v>1.043426375803417</v>
       </c>
       <c r="C9">
-        <v>0.6933101177503062</v>
+        <v>0.807206677788961</v>
       </c>
       <c r="D9">
-        <v>0.7359835305854562</v>
+        <v>0.6305252804930227</v>
       </c>
       <c r="E9">
-        <v>0.7673968131939678</v>
+        <v>0.5351760848342041</v>
       </c>
     </row>
     <row r="10" spans="1:5">
@@ -521,16 +521,16 @@
         <v>9</v>
       </c>
       <c r="B10">
-        <v>0.5751234693798278</v>
+        <v>0.1446119706244076</v>
       </c>
       <c r="C10">
-        <v>0.7155094639707574</v>
+        <v>0.1778433927788587</v>
       </c>
       <c r="D10">
-        <v>0.7610162011337268</v>
+        <v>0.1913537846781337</v>
       </c>
       <c r="E10">
-        <v>0.7856474367023336</v>
+        <v>0.1952765305098286</v>
       </c>
     </row>
     <row r="11" spans="1:5">
@@ -538,16 +538,16 @@
         <v>10</v>
       </c>
       <c r="B11">
-        <v>0.5761168760917758</v>
+        <v>0.1486753228623937</v>
       </c>
       <c r="C11">
-        <v>0.7140132558073445</v>
+        <v>0.172745142534035</v>
       </c>
       <c r="D11">
-        <v>0.7627958820574808</v>
+        <v>0.1845473908203582</v>
       </c>
       <c r="E11">
-        <v>0.7898377149511048</v>
+        <v>0.2038290877293174</v>
       </c>
     </row>
     <row r="12" spans="1:5">
@@ -555,16 +555,16 @@
         <v>11</v>
       </c>
       <c r="B12">
-        <v>0.6352131230705311</v>
+        <v>0.5908383472761032</v>
       </c>
       <c r="C12">
-        <v>0.7313851181014966</v>
+        <v>0.6258712075917138</v>
       </c>
       <c r="D12">
-        <v>0.759398913530363</v>
+        <v>0.7677355432521035</v>
       </c>
       <c r="E12">
-        <v>0.7812697644724856</v>
+        <v>1.023780436895768</v>
       </c>
     </row>
     <row r="13" spans="1:5">
@@ -572,16 +572,16 @@
         <v>12</v>
       </c>
       <c r="B13">
-        <v>0.5719969355166875</v>
+        <v>0.1437325632836805</v>
       </c>
       <c r="C13">
-        <v>0.7108772263761759</v>
+        <v>0.174985163415674</v>
       </c>
       <c r="D13">
-        <v>0.7590621141496083</v>
+        <v>0.1907386850940041</v>
       </c>
       <c r="E13">
-        <v>0.7838646314813464</v>
+        <v>0.1969711125260819</v>
       </c>
     </row>
   </sheetData>

</xml_diff>